<commit_message>
feat: skip words Tân already knows
known-words.txt is his own list, one word per line, and nothing on it becomes a card.

It is checked in two places on purpose. A SessionStart hook prints the list into the
session, so the answer does not spend one of its three word-list slots on a word he has;
and vocab-capture.py checks the same file before queueing, which is the half that still
works when the answer is written without looking. The first saves a slot, the second is
the guarantee.

Matching is the whole line, lower-cased, with no stemming: one line covers every part of
speech of a word, and nothing is silenced by accident.

Adding a word does not remove the row it already has. The sheet is rebuilt from
history.jsonl, which records what was taught, and a card already in Anki carries review
history worth more than the tidiness of deleting it.
</commit_message>
<xml_diff>
--- a/my-vocab-sheet.xlsx
+++ b/my-vocab-sheet.xlsx
@@ -1525,10 +1525,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;#xFF2D;&amp;amp;amp;#xFF33; &amp;amp;amp;#xFF30;&amp;amp;amp;#x30B4;&amp;amp;amp;#x30B7;&amp;amp;amp;#x30C3;&amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;#xB9D1;&amp;amp;amp;#xC740; &amp;amp;amp;#xACE0;&amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;#x5B8B;&amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;#x65B0;&amp;amp;amp;#x7D30;&amp;amp;amp;#x660E;&amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1559,10 +1559,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;#xFF2D;&amp;amp;amp;#xFF33; &amp;amp;amp;#xFF30;&amp;amp;amp;#x30B4;&amp;amp;amp;#x30B7;&amp;amp;amp;#x30C3;&amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;#xB9D1;&amp;amp;amp;#xC740; &amp;amp;amp;#xACE0;&amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;#x5B8B;&amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;#x65B0;&amp;amp;amp;#x7D30;&amp;amp;amp;#x660E;&amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1763,7 +1763,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{591C8CB4-E913-44F9-A63C-4B9162A9CB95}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EF33030A-EBA7-4F3F-9965-36B37909BD81}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I73"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -3761,7 +3761,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{313311BC-A14D-49C1-9F09-8E6EDB9E868F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0C339DC9-8E53-4FFE-9B62-72A8FC77E3B0}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>

</xml_diff>